<commit_message>
Refresh Returns & Refunds data (2026-08-22–2026-08-28)
Add new ASIN B0HFQ5HGX3 (Organic Argan Oil) as EO-ARGAN-Master family.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SK9y9ywmPoJtSWqM5ZTvh1
</commit_message>
<xml_diff>
--- a/bodyj4you-return-dashboard/data/catalog.xlsx
+++ b/bodyj4you-return-dashboard/data/catalog.xlsx
@@ -1211,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F215"/>
+  <dimension ref="A1:F216"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="29.36328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="26.54296875" bestFit="1" customWidth="1" style="101" min="1" max="1"/>
@@ -8012,6 +8012,34 @@
         </is>
       </c>
       <c r="F215" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>EO-ARGAN-1oz</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>B0HFQ5HGX3</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>EO-ARGAN-Master</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>EO</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr">
         <is>
           <t>Miami</t>
         </is>

</xml_diff>

<commit_message>
Refresh Returns & Refunds data (2026-08-23–2026-08-29)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPB9SrSKAcK8oR7iKrMaBd
</commit_message>
<xml_diff>
--- a/bodyj4you-return-dashboard/data/catalog.xlsx
+++ b/bodyj4you-return-dashboard/data/catalog.xlsx
@@ -1211,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F216"/>
+  <dimension ref="A1:F217"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="29.36328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="26.54296875" bestFit="1" customWidth="1" style="101" min="1" max="1"/>
@@ -8038,8 +8038,39 @@
           <t>EO</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>PD-TEATREE-MCT-Spray</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>B0HFMFM9BD</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>PD-TEATREE-MCT-Master</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>EO</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>PD-TEATREE-MCT-Spray</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
         <is>
           <t>Miami</t>
         </is>

</xml_diff>

<commit_message>
Refresh Returns & Refunds data (2026-09-02–2026-09-08)
Catalog: added B0HFBPRVLR (2PC Rainbow Choker) to NC4285-Master.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LX6kCTHJkv83K6EszcHMEQ
</commit_message>
<xml_diff>
--- a/bodyj4you-return-dashboard/data/catalog.xlsx
+++ b/bodyj4you-return-dashboard/data/catalog.xlsx
@@ -1211,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F217"/>
+  <dimension ref="A1:F218"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="29.36328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="26.54296875" bestFit="1" customWidth="1" style="101" min="1" max="1"/>
@@ -8073,6 +8073,33 @@
       <c r="F217" t="inlineStr">
         <is>
           <t>Miami</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>B0HFBPRVLR</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>B0HFBPRVLR</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>NC4285-Master</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>China</t>
         </is>
       </c>
     </row>

</xml_diff>